<commit_message>
New sample run with peer review.
</commit_message>
<xml_diff>
--- a/sample-data/sample-run/Tech Review.xlsx
+++ b/sample-data/sample-run/Tech Review.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>43 cell(s) &gt; 1.0</t>
+          <t>136 cell(s) &gt; 1.0</t>
         </is>
       </c>
     </row>
@@ -913,7 +913,7 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>13 period(s): ['period 3: 46%', 'period 4: 101%', 'period 6: 244%']</t>
+          <t>13 period(s): ['period 3: 45%', 'period 4: 101%', 'period 6: 244%']</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>43 cell(s) &gt; 1.0</t>
+          <t>136 cell(s) &gt; 1.0</t>
         </is>
       </c>
     </row>
@@ -1543,7 +1543,7 @@
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>Median=4,773</t>
+          <t>Median=4,584</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>13 period(s): ['period 3: 46%', 'period 4: 101%', 'period 6: 244%']</t>
+          <t>13 period(s): ['period 3: 45%', 'period 4: 101%', 'period 6: 244%']</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Address issues mentioned in peer review from latest sample run.
</commit_message>
<xml_diff>
--- a/sample-data/sample-run/Tech Review.xlsx
+++ b/sample-data/sample-run/Tech Review.xlsx
@@ -490,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -529,127 +529,127 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>1. Structure</t>
+          <t>2. Period Consistency</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Measure sheets present</t>
+          <t>'Incurred-to-Ult' periods match measures</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>None of: Incurred Loss, Paid Loss, Reported Count, Closed Count</t>
+          <t>missing: {'Total'}</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>2. Period Consistency</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>Period consistency</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>No measure sheets — skipping</t>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>'Paid-to-Ult' periods match measures</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>missing: {'Total'}</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>3. Current Age / Maturity</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Maturity checks</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>No measure sheets — skipping</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>2. Period Consistency</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>'Reported-to-Ult' periods match measures</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>missing: {'Total'}</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>6. Sel - Sheet Consistency</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>Sel - sheets present</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>4. Selected Ultimate Integrity</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>'Loss Selection' no null Selected Ultimates</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>1 null(s)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>7. X-to-Ult Triangles</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>'Incurred-to-Ult' all values in (0, 1]</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>16 cell(s) &gt; 1.0</t>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>4. Selected Ultimate Integrity</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>'Loss Selection' IBNR &gt;= 0</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Below tolerance in periods: ['2001', '2002', '2006', '2012']</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>7. X-to-Ult Triangles</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>'Incurred-to-Ult' non-decreasing across ages</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>31 reversal(s)</t>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>4. Selected Ultimate Integrity</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>'Count Selection' no null Selected Ultimates</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>1 null(s)</t>
         </is>
       </c>
     </row>
@@ -661,17 +661,17 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>7. X-to-Ult Triangles</t>
+          <t>4. Selected Ultimate Integrity</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>'Paid-to-Ult' non-decreasing across ages</t>
+          <t>'Count Selection' IBNR &gt;= 0</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>5 reversal(s)</t>
+          <t>Slight negatives (within tolerance) periods: ['2002', '2003', '2008', '2009', '2012', '2013', '2014', '2016', '2017', '2018', '2019', '2020', '2021', '2022', '2023']</t>
         </is>
       </c>
     </row>
@@ -683,39 +683,39 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
+          <t>6. Sel - Sheet Consistency</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Sel - sheets present</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
           <t>7. X-to-Ult Triangles</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>'Reported-to-Ult' all values in (0, 1]</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>136 cell(s) &gt; 1.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>7. X-to-Ult Triangles</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>'Reported-to-Ult' non-decreasing across ages</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>6 reversal(s)</t>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>'Incurred-to-Ult' row count = period count</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Triangle=24, Measures=25</t>
         </is>
       </c>
     </row>
@@ -727,17 +727,17 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>8. Average IBNR / Unpaid</t>
+          <t>7. X-to-Ult Triangles</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Average IBNR all values &gt;= 0</t>
+          <t>'Incurred-to-Ult' all values in (0, 1]</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>16 cell(s) &lt; 0</t>
+          <t>16 cell(s) &gt; 1.0</t>
         </is>
       </c>
     </row>
@@ -749,12 +749,12 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>8. Average IBNR / Unpaid</t>
+          <t>7. X-to-Ult Triangles</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Average IBNR non-increasing across ages</t>
+          <t>'Incurred-to-Ult' non-decreasing across ages</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -764,24 +764,24 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>8. Average IBNR / Unpaid</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>Average Unpaid non-increasing across ages</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>5 reversal(s)</t>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>7. X-to-Ult Triangles</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>'Paid-to-Ult' row count = period count</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Triangle=24, Measures=25</t>
         </is>
       </c>
     </row>
@@ -793,39 +793,39 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>10. CL Triangle Integrity</t>
+          <t>7. X-to-Ult Triangles</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>CL triangles present</t>
+          <t>'Paid-to-Ult' non-decreasing across ages</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
+          <t>5 reversal(s)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>11. Development Factors</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>Development factor checks</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>7. X-to-Ult Triangles</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>'Reported-to-Ult' row count = period count</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Triangle=24, Measures=25</t>
         </is>
       </c>
     </row>
@@ -837,17 +837,17 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>12. Paid-to-Incurred Raw Data</t>
+          <t>7. X-to-Ult Triangles</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Paid and Incurred present</t>
+          <t>'Reported-to-Ult' all values in (0, 1]</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>One or both missing — skipping</t>
+          <t>136 cell(s) &gt; 1.0</t>
         </is>
       </c>
     </row>
@@ -859,17 +859,17 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>13. Case Reserve Reasonableness</t>
+          <t>7. X-to-Ult Triangles</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Case reserves check</t>
+          <t>'Reported-to-Ult' non-decreasing across ages</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Incurred Loss and/or Paid Loss missing — skipping</t>
+          <t>6 reversal(s)</t>
         </is>
       </c>
     </row>
@@ -881,17 +881,17 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>14. Closure Rate Checks</t>
+          <t>8. Average IBNR / Unpaid</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Closure rate checks</t>
+          <t>Average IBNR all values &gt;= 0</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Reported Count and/or Closed Count missing — skipping</t>
+          <t>16 cell(s) &lt; 0</t>
         </is>
       </c>
     </row>
@@ -903,17 +903,17 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>15. Severity / Frequency Trends</t>
+          <t>8. Average IBNR / Unpaid</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>YoY severity change &gt; 25% detected</t>
+          <t>Average IBNR non-increasing across ages</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>13 period(s): ['period 3: 45%', 'period 4: 101%', 'period 6: 244%']</t>
+          <t>31 reversal(s)</t>
         </is>
       </c>
     </row>
@@ -925,15 +925,169 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
+          <t>8. Average IBNR / Unpaid</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Average Unpaid non-increasing across ages</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>5 reversal(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>10. CL Triangle Integrity</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>CL triangles present</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>11. Development Factors</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Development factor checks</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>12. Paid-to-Incurred Raw Data</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Paid and Incurred present</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>One or both missing — skipping</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>13. Case Reserve Reasonableness</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Case reserves check</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Incurred Loss and/or Paid Loss missing — skipping</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>14. Closure Rate Checks</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Closure rate checks</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Reported Count and/or Closed Count missing — skipping</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
           <t>15. Severity / Frequency Trends</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>YoY severity change &gt; 25% detected</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>13 period(s): ['period 3: 45%', 'period 4: 101%', 'period 6: 244%']</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>15. Severity / Frequency Trends</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>Frequency spike &gt; 2x median detected</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>5 period(s) above 2x median (0.0000)</t>
         </is>
@@ -950,7 +1104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1004,24 +1158,24 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>1. Structure</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>Measure sheets present</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>None of: Incurred Loss, Paid Loss, Reported Count, Closed Count</t>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>Loss Selection, Count Selection</t>
         </is>
       </c>
     </row>
@@ -1084,134 +1238,130 @@
       <c r="D6" s="10" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>2. Period Consistency</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Period consistency</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>No measure sheets — skipping</t>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>All measure sheets same periods</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>25 periods</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>3. Current Age / Maturity</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Maturity checks</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>No measure sheets — skipping</t>
-        </is>
-      </c>
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>2. Period Consistency</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Diagnostics periods in measure periods</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>6. Sel - Sheet Consistency</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>Sel - sheets present</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>2. Period Consistency</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>'Incurred-to-Ult' periods match measures</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>missing: {'Total'}</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>7. X-to-Ult Triangles</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>'Incurred-to-Ult' all values in (0, 1]</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>16 cell(s) &gt; 1.0</t>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>2. Period Consistency</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>'Paid-to-Ult' periods match measures</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>missing: {'Total'}</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>7. X-to-Ult Triangles</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>'Incurred-to-Ult' most-mature diagonal ~= 1.0</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="inlineStr">
-        <is>
-          <t>1.0359</t>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>2. Period Consistency</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>'Reported-to-Ult' periods match measures</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>missing: {'Total'}</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>7. X-to-Ult Triangles</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>'Incurred-to-Ult' non-decreasing across ages</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>31 reversal(s)</t>
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>2. Period Consistency</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Period sequence (non-integer — consecutive check skipped)</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>25 periods</t>
         </is>
       </c>
     </row>
@@ -1223,12 +1373,12 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>7. X-to-Ult Triangles</t>
+          <t>3. Current Age / Maturity</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>'Paid-to-Ult' all values in (0, 1]</t>
+          <t>All current ages &gt; 0</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr"/>
@@ -1241,61 +1391,61 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>7. X-to-Ult Triangles</t>
+          <t>3. Current Age / Maturity</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>'Paid-to-Ult' most-mature diagonal ~= 1.0</t>
+          <t>All current ages multiples of 12</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>0.9961</t>
+          <t>11-month development pattern detected (ages 11, 23, 35, ...) — valid</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>7. X-to-Ult Triangles</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>'Paid-to-Ult' non-decreasing across ages</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>5 reversal(s)</t>
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>3. Current Age / Maturity</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Max current age within range</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>287</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>7. X-to-Ult Triangles</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>'Reported-to-Ult' all values in (0, 1]</t>
-        </is>
-      </c>
-      <c r="D16" s="7" t="inlineStr">
-        <is>
-          <t>136 cell(s) &gt; 1.0</t>
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>3. Current Age / Maturity</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Min current age &gt;= 11</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>11</t>
         </is>
       </c>
     </row>
@@ -1307,39 +1457,35 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>7. X-to-Ult Triangles</t>
+          <t>3. Current Age / Maturity</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>'Reported-to-Ult' most-mature diagonal ~= 1.0</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
-      </c>
+          <t>Maturity ordering (non-integer periods — order check skipped)</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>7. X-to-Ult Triangles</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>'Reported-to-Ult' non-decreasing across ages</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t>6 reversal(s)</t>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>4. Selected Ultimate Integrity</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>'Loss Selection' no null Selected Ultimates</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>1 null(s)</t>
         </is>
       </c>
     </row>
@@ -1351,79 +1497,75 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>7. X-to-Ult Triangles</t>
+          <t>4. Selected Ultimate Integrity</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>Incurred-to-Ult &gt;= Paid-to-Ult at all cells</t>
+          <t>'Loss Selection' all Selected Ultimates &gt; 0</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>8. Average IBNR / Unpaid</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>Average IBNR all values &gt;= 0</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t>16 cell(s) &lt; 0</t>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>4. Selected Ultimate Integrity</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>'Loss Selection' IBNR &gt;= 0</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Below tolerance in periods: ['2001', '2002', '2006', '2012']</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>8. Average IBNR / Unpaid</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>Average IBNR non-increasing across ages</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>31 reversal(s)</t>
-        </is>
-      </c>
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>4. Selected Ultimate Integrity</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>'Loss Selection' no extreme outlier ultimates</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>8. Average IBNR / Unpaid</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>Average IBNR most-mature period final value ~= 0</t>
-        </is>
-      </c>
-      <c r="D22" s="10" t="inlineStr">
-        <is>
-          <t>-109,614</t>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>4. Selected Ultimate Integrity</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>'Count Selection' no null Selected Ultimates</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>1 null(s)</t>
         </is>
       </c>
     </row>
@@ -1435,12 +1577,12 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>8. Average IBNR / Unpaid</t>
+          <t>4. Selected Ultimate Integrity</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>Average Unpaid all values &gt;= 0</t>
+          <t>'Count Selection' all Selected Ultimates &gt; 0</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr"/>
@@ -1453,17 +1595,17 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>8. Average IBNR / Unpaid</t>
+          <t>4. Selected Ultimate Integrity</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Average Unpaid non-increasing across ages</t>
+          <t>'Count Selection' IBNR &gt;= 0</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>5 reversal(s)</t>
+          <t>Slight negatives (within tolerance) periods: ['2002', '2003', '2008', '2009', '2012', '2013', '2014', '2016', '2017', '2018', '2019', '2020', '2021', '2022', '2023']</t>
         </is>
       </c>
     </row>
@@ -1475,75 +1617,79 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>8. Average IBNR / Unpaid</t>
+          <t>4. Selected Ultimate Integrity</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>Average Unpaid most-mature period final value ~= 0</t>
-        </is>
-      </c>
-      <c r="D25" s="10" t="inlineStr">
-        <is>
-          <t>11,865</t>
-        </is>
-      </c>
+          <t>'Count Selection' no extreme outlier ultimates</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>8. Average IBNR / Unpaid</t>
-        </is>
-      </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>Average Unpaid &gt;= Average IBNR at all matching cells</t>
-        </is>
-      </c>
-      <c r="D26" s="10" t="inlineStr"/>
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>6. Sel - Sheet Consistency</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>Sel - sheets present</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>9. Diagnostics</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>Ultimate Severity &gt; 0 for all periods</t>
-        </is>
-      </c>
-      <c r="D27" s="10" t="inlineStr"/>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>7. X-to-Ult Triangles</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>'Incurred-to-Ult' row count = period count</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Triangle=24, Measures=25</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>9. Diagnostics</t>
-        </is>
-      </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>Ultimate Severity no outliers</t>
-        </is>
-      </c>
-      <c r="D28" s="10" t="inlineStr">
-        <is>
-          <t>Median=4,584</t>
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>7. X-to-Ult Triangles</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>'Incurred-to-Ult' all values in (0, 1]</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>16 cell(s) &gt; 1.0</t>
         </is>
       </c>
     </row>
@@ -1555,101 +1701,101 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>9. Diagnostics</t>
+          <t>7. X-to-Ult Triangles</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>Loss Rate in (0, 2.0)</t>
+          <t>'Incurred-to-Ult' most-mature diagonal ~= 1.0</t>
         </is>
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>Range: 0.002-0.014</t>
+          <t>1.0359</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>9. Diagnostics</t>
-        </is>
-      </c>
-      <c r="C30" s="9" t="inlineStr">
-        <is>
-          <t>Ultimate Frequency &gt; 0 for all periods</t>
-        </is>
-      </c>
-      <c r="D30" s="10" t="inlineStr"/>
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>7. X-to-Ult Triangles</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>'Incurred-to-Ult' non-decreasing across ages</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>31 reversal(s)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t>10. CL Triangle Integrity</t>
-        </is>
-      </c>
-      <c r="C31" s="6" t="inlineStr">
-        <is>
-          <t>CL triangles present</t>
-        </is>
-      </c>
-      <c r="D31" s="7" t="inlineStr">
-        <is>
-          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>7. X-to-Ult Triangles</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>'Paid-to-Ult' row count = period count</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Triangle=24, Measures=25</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>11. Development Factors</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="inlineStr">
-        <is>
-          <t>Development factor checks</t>
-        </is>
-      </c>
-      <c r="D32" s="7" t="inlineStr">
-        <is>
-          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
-        </is>
-      </c>
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>7. X-to-Ult Triangles</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>'Paid-to-Ult' all values in (0, 1]</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B33" s="6" t="inlineStr">
-        <is>
-          <t>12. Paid-to-Incurred Raw Data</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="inlineStr">
-        <is>
-          <t>Paid and Incurred present</t>
-        </is>
-      </c>
-      <c r="D33" s="7" t="inlineStr">
-        <is>
-          <t>One or both missing — skipping</t>
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>7. X-to-Ult Triangles</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>'Paid-to-Ult' most-mature diagonal ~= 1.0</t>
+        </is>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t>0.9961</t>
         </is>
       </c>
     </row>
@@ -1661,39 +1807,39 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>13. Case Reserve Reasonableness</t>
+          <t>7. X-to-Ult Triangles</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Case reserves check</t>
+          <t>'Paid-to-Ult' non-decreasing across ages</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>Incurred Loss and/or Paid Loss missing — skipping</t>
+          <t>5 reversal(s)</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B35" s="6" t="inlineStr">
-        <is>
-          <t>14. Closure Rate Checks</t>
-        </is>
-      </c>
-      <c r="C35" s="6" t="inlineStr">
-        <is>
-          <t>Closure rate checks</t>
-        </is>
-      </c>
-      <c r="D35" s="7" t="inlineStr">
-        <is>
-          <t>Reported Count and/or Closed Count missing — skipping</t>
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>7. X-to-Ult Triangles</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>'Reported-to-Ult' row count = period count</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Triangle=24, Measures=25</t>
         </is>
       </c>
     </row>
@@ -1705,37 +1851,457 @@
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
+          <t>7. X-to-Ult Triangles</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>'Reported-to-Ult' all values in (0, 1]</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>136 cell(s) &gt; 1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>7. X-to-Ult Triangles</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="inlineStr">
+        <is>
+          <t>'Reported-to-Ult' most-mature diagonal ~= 1.0</t>
+        </is>
+      </c>
+      <c r="D37" s="10" t="inlineStr">
+        <is>
+          <t>1.0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>7. X-to-Ult Triangles</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>'Reported-to-Ult' non-decreasing across ages</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>6 reversal(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>7. X-to-Ult Triangles</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>Incurred-to-Ult &gt;= Paid-to-Ult at all cells</t>
+        </is>
+      </c>
+      <c r="D39" s="10" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>8. Average IBNR / Unpaid</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>Average IBNR all values &gt;= 0</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>16 cell(s) &lt; 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>8. Average IBNR / Unpaid</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Average IBNR non-increasing across ages</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>31 reversal(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>8. Average IBNR / Unpaid</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>Average IBNR most-mature period final value ~= 0</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>-109,614</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>8. Average IBNR / Unpaid</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>Average Unpaid all values &gt;= 0</t>
+        </is>
+      </c>
+      <c r="D43" s="10" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>8. Average IBNR / Unpaid</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>Average Unpaid non-increasing across ages</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>5 reversal(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>8. Average IBNR / Unpaid</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>Average Unpaid most-mature period final value ~= 0</t>
+        </is>
+      </c>
+      <c r="D45" s="10" t="inlineStr">
+        <is>
+          <t>11,865</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>8. Average IBNR / Unpaid</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>Average Unpaid &gt;= Average IBNR at all matching cells</t>
+        </is>
+      </c>
+      <c r="D46" s="10" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>9. Diagnostics</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>Ultimate Severity &gt; 0 for all periods</t>
+        </is>
+      </c>
+      <c r="D47" s="10" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>9. Diagnostics</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>Ultimate Severity no outliers</t>
+        </is>
+      </c>
+      <c r="D48" s="10" t="inlineStr">
+        <is>
+          <t>Median=4,584</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>9. Diagnostics</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="inlineStr">
+        <is>
+          <t>Loss Rate in (0, 2.0)</t>
+        </is>
+      </c>
+      <c r="D49" s="10" t="inlineStr">
+        <is>
+          <t>Range: 0.002-0.014</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>9. Diagnostics</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>Ultimate Frequency &gt; 0 for all periods</t>
+        </is>
+      </c>
+      <c r="D50" s="10" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>10. CL Triangle Integrity</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>CL triangles present</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>11. Development Factors</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>Development factor checks</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>12. Paid-to-Incurred Raw Data</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>Paid and Incurred present</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>One or both missing — skipping</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>13. Case Reserve Reasonableness</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>Case reserves check</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>Incurred Loss and/or Paid Loss missing — skipping</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>14. Closure Rate Checks</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>Closure rate checks</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>Reported Count and/or Closed Count missing — skipping</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
           <t>15. Severity / Frequency Trends</t>
         </is>
       </c>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="C56" s="6" t="inlineStr">
         <is>
           <t>YoY severity change &gt; 25% detected</t>
         </is>
       </c>
-      <c r="D36" s="7" t="inlineStr">
+      <c r="D56" s="7" t="inlineStr">
         <is>
           <t>13 period(s): ['period 3: 45%', 'period 4: 101%', 'period 6: 244%']</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B37" s="6" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
         <is>
           <t>15. Severity / Frequency Trends</t>
         </is>
       </c>
-      <c r="C37" s="6" t="inlineStr">
+      <c r="C57" s="6" t="inlineStr">
         <is>
           <t>Frequency spike &gt; 2x median detected</t>
         </is>
       </c>
-      <c r="D37" s="7" t="inlineStr">
+      <c r="D57" s="7" t="inlineStr">
         <is>
           <t>5 period(s) above 2x median (0.0000)</t>
         </is>

</xml_diff>

<commit_message>
New sample run from scratch.
</commit_message>
<xml_diff>
--- a/sample-data/sample-run/Tech Review.xlsx
+++ b/sample-data/sample-run/Tech Review.xlsx
@@ -490,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -534,34 +534,34 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
+          <t>Diagnostics sheet present</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>1. Structure</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
           <t>X-to-Ult triangle sheets present</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>4. Selected Ultimate Integrity</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>'Loss Selection' no null Selected Ultimates</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>1 null(s)</t>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
         </is>
       </c>
     </row>
@@ -578,12 +578,12 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>'Count Selection' no null Selected Ultimates</t>
+          <t>'Loss Selection' IBNR &gt;= 0</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>1 null(s)</t>
+          <t>Below tolerance in periods: ['2001', '2002', '2006', '2012']</t>
         </is>
       </c>
     </row>
@@ -600,12 +600,12 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>'Count Selection' IBNR &gt;= 0</t>
+          <t>'Loss Selection' no extreme outlier ultimates</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Slight negatives (within tolerance) periods: ['2002', '2003', '2008', '2009', '2012', '2013', '2014', '2016', '2018']</t>
+          <t>1 period(s) &gt; 10.0x median (1,708,556)</t>
         </is>
       </c>
     </row>
@@ -617,17 +617,17 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>6. Sel - Sheet Consistency</t>
+          <t>4. Selected Ultimate Integrity</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Sel - sheets present</t>
+          <t>'Count Selection' IBNR &gt;= 0</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
+          <t>Slight negatives (within tolerance) periods: ['2002', '2003', '2008', '2009', '2012', '2013', '2014', '2016', '2017', '2018', '2019', '2020', '2021', '2022', '2023']</t>
         </is>
       </c>
     </row>
@@ -639,17 +639,17 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>7. X-to-Ult Triangles</t>
+          <t>4. Selected Ultimate Integrity</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>X-to-Ult triangles</t>
+          <t>'Count Selection' no extreme outlier ultimates</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
+          <t>1 period(s) &gt; 10.0x median (346)</t>
         </is>
       </c>
     </row>
@@ -661,12 +661,12 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>8. Average IBNR / Unpaid</t>
+          <t>6. Sel - Sheet Consistency</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Average IBNR has data</t>
+          <t>Sel - sheets present</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -683,12 +683,12 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>8. Average IBNR / Unpaid</t>
+          <t>7. X-to-Ult Triangles</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Average Unpaid has data</t>
+          <t>X-to-Ult triangles</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -705,12 +705,12 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>10. CL Triangle Integrity</t>
+          <t>8. Average IBNR / Unpaid</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>CL triangles present</t>
+          <t>Average IBNR has data</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -727,12 +727,12 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>11. Development Factors</t>
+          <t>8. Average IBNR / Unpaid</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Development factor checks</t>
+          <t>Average Unpaid has data</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -749,17 +749,17 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>12. Paid-to-Incurred Raw Data</t>
+          <t>9. Diagnostics</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Paid and Incurred present</t>
+          <t>Diagnostics</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>One or both missing — skipping</t>
+          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
         </is>
       </c>
     </row>
@@ -771,17 +771,17 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>13. Case Reserve Reasonableness</t>
+          <t>10. CL Triangle Integrity</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Case reserves check</t>
+          <t>CL triangles present</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Incurred Loss and/or Paid Loss missing — skipping</t>
+          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
         </is>
       </c>
     </row>
@@ -793,17 +793,17 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>14. Closure Rate Checks</t>
+          <t>11. Development Factors</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Closure rate checks</t>
+          <t>Development factor checks</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Reported Count and/or Closed Count missing — skipping</t>
+          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
         </is>
       </c>
     </row>
@@ -815,17 +815,17 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>15. Severity / Frequency Trends</t>
+          <t>12. Paid-to-Incurred Raw Data</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>YoY severity change &gt; 25% detected</t>
+          <t>Paid and Incurred present</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>13 period(s): ['period 3: 46%', 'period 4: 103%', 'period 6: 231%']</t>
+          <t>One or both missing — skipping</t>
         </is>
       </c>
     </row>
@@ -837,17 +837,61 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
+          <t>13. Case Reserve Reasonableness</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Case reserves check</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Incurred Loss and/or Paid Loss missing — skipping</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>14. Closure Rate Checks</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Closure rate checks</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Reported Count and/or Closed Count missing — skipping</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
           <t>15. Severity / Frequency Trends</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>Frequency spike &gt; 2x median detected</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>5 period(s) above 2x median (0.0000)</t>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Trend checks</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Diagnostics sheet missing — skipping</t>
         </is>
       </c>
     </row>
@@ -862,7 +906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -911,7 +955,7 @@
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>16 sheets</t>
+          <t>15 sheets</t>
         </is>
       </c>
     </row>
@@ -938,22 +982,26 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>1. Structure</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Diagnostics sheet present</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr"/>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1030,10 +1078,14 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Diagnostics periods in measure periods</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="inlineStr"/>
+          <t>Period sequence (non-integer — consecutive check skipped)</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>25 periods</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
@@ -1043,19 +1095,15 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>2. Period Consistency</t>
+          <t>3. Current Age / Maturity</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Period sequence (non-integer — consecutive check skipped)</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="inlineStr">
-        <is>
-          <t>25 periods</t>
-        </is>
-      </c>
+          <t>All current ages &gt; 0</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -1070,10 +1118,14 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>All current ages &gt; 0</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="inlineStr"/>
+          <t>All current ages multiples of 12</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>11-month development pattern detected (ages 11, 23, 35, ...) — valid</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -1088,12 +1140,12 @@
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>All current ages multiples of 12</t>
+          <t>Max current age within range</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>11-month development pattern detected (ages 11, 23, 35, ...) — valid</t>
+          <t>287</t>
         </is>
       </c>
     </row>
@@ -1110,12 +1162,12 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Max current age within range</t>
+          <t>Min current age &gt;= 11</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>287</t>
+          <t>11</t>
         </is>
       </c>
     </row>
@@ -1132,14 +1184,10 @@
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>Min current age &gt;= 11</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
+          <t>Maturity ordering (non-integer periods — order check skipped)</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -1149,73 +1197,77 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>3. Current Age / Maturity</t>
+          <t>4. Selected Ultimate Integrity</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>Maturity ordering (non-integer periods — order check skipped)</t>
+          <t>'Loss Selection' no null Selected Ultimates</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>4. Selected Ultimate Integrity</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>'Loss Selection' all Selected Ultimates &gt; 0</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>4. Selected Ultimate Integrity</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>'Loss Selection' no null Selected Ultimates</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>1 null(s)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>'Loss Selection' IBNR &gt;= 0</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Below tolerance in periods: ['2001', '2002', '2006', '2012']</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>4. Selected Ultimate Integrity</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>'Loss Selection' all Selected Ultimates &gt; 0</t>
-        </is>
-      </c>
-      <c r="D16" s="10" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>4. Selected Ultimate Integrity</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>'Loss Selection' IBNR &gt;= 0</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="inlineStr"/>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>'Loss Selection' no extreme outlier ultimates</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>1 period(s) &gt; 10.0x median (1,708,556)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
@@ -1230,50 +1282,50 @@
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>'Loss Selection' no extreme outlier ultimates</t>
+          <t>'Count Selection' no null Selected Ultimates</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>4. Selected Ultimate Integrity</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>'Count Selection' no null Selected Ultimates</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>1 null(s)</t>
-        </is>
-      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>'Count Selection' all Selected Ultimates &gt; 0</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>4. Selected Ultimate Integrity</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>'Count Selection' all Selected Ultimates &gt; 0</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr"/>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>'Count Selection' IBNR &gt;= 0</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Slight negatives (within tolerance) periods: ['2002', '2003', '2008', '2009', '2012', '2013', '2014', '2016', '2017', '2018', '2019', '2020', '2021', '2022', '2023']</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1288,32 +1340,36 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>'Count Selection' IBNR &gt;= 0</t>
+          <t>'Count Selection' no extreme outlier ultimates</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Slight negatives (within tolerance) periods: ['2002', '2003', '2008', '2009', '2012', '2013', '2014', '2016', '2018']</t>
+          <t>1 period(s) &gt; 10.0x median (346)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>4. Selected Ultimate Integrity</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>'Count Selection' no extreme outlier ultimates</t>
-        </is>
-      </c>
-      <c r="D22" s="10" t="inlineStr"/>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>6. Sel - Sheet Consistency</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Sel - sheets present</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1323,12 +1379,12 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>6. Sel - Sheet Consistency</t>
+          <t>7. X-to-Ult Triangles</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Sel - sheets present</t>
+          <t>X-to-Ult triangles</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -1345,12 +1401,12 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>7. X-to-Ult Triangles</t>
+          <t>8. Average IBNR / Unpaid</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>X-to-Ult triangles</t>
+          <t>Average IBNR has data</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -1372,7 +1428,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Average IBNR has data</t>
+          <t>Average Unpaid has data</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -1389,12 +1445,12 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>8. Average IBNR / Unpaid</t>
+          <t>9. Diagnostics</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Average Unpaid has data</t>
+          <t>Diagnostics</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -1404,84 +1460,92 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>9. Diagnostics</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>Ultimate Severity &gt; 0 for all periods</t>
-        </is>
-      </c>
-      <c r="D27" s="10" t="inlineStr"/>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>10. CL Triangle Integrity</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>CL triangles present</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>9. Diagnostics</t>
-        </is>
-      </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>Ultimate Severity no outliers</t>
-        </is>
-      </c>
-      <c r="D28" s="10" t="inlineStr">
-        <is>
-          <t>Median=4,476</t>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>11. Development Factors</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Development factor checks</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>9. Diagnostics</t>
-        </is>
-      </c>
-      <c r="C29" s="9" t="inlineStr">
-        <is>
-          <t>Loss Rate in (0, 2.0)</t>
-        </is>
-      </c>
-      <c r="D29" s="10" t="inlineStr">
-        <is>
-          <t>Range: 0.002-0.014</t>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>12. Paid-to-Incurred Raw Data</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Paid and Incurred present</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>One or both missing — skipping</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>9. Diagnostics</t>
-        </is>
-      </c>
-      <c r="C30" s="9" t="inlineStr">
-        <is>
-          <t>Ultimate Frequency &gt; 0 for all periods</t>
-        </is>
-      </c>
-      <c r="D30" s="10" t="inlineStr"/>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>13. Case Reserve Reasonableness</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Case reserves check</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Incurred Loss and/or Paid Loss missing — skipping</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1491,17 +1555,17 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>10. CL Triangle Integrity</t>
+          <t>14. Closure Rate Checks</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>CL triangles present</t>
+          <t>Closure rate checks</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
+          <t>Reported Count and/or Closed Count missing — skipping</t>
         </is>
       </c>
     </row>
@@ -1513,127 +1577,17 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>11. Development Factors</t>
+          <t>15. Severity / Frequency Trends</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Development factor checks</t>
+          <t>Trend checks</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Not in values file — see complete-analysis.xlsx (expected)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>12. Paid-to-Incurred Raw Data</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>Paid and Incurred present</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>One or both missing — skipping</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>13. Case Reserve Reasonableness</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>Case reserves check</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>Incurred Loss and/or Paid Loss missing — skipping</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>14. Closure Rate Checks</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>Closure rate checks</t>
-        </is>
-      </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>Reported Count and/or Closed Count missing — skipping</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>15. Severity / Frequency Trends</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>YoY severity change &gt; 25% detected</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>13 period(s): ['period 3: 46%', 'period 4: 103%', 'period 6: 231%']</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>15. Severity / Frequency Trends</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>Frequency spike &gt; 2x median detected</t>
-        </is>
-      </c>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>5 period(s) above 2x median (0.0000)</t>
+          <t>Diagnostics sheet missing — skipping</t>
         </is>
       </c>
     </row>

</xml_diff>